<commit_message>
Add LDS 3.0 tab and clean up names and jargon on LDS dashboard
LDS 3.0 is a separate program with different attendees, so it gets its
own page and data file instead of being merged into the prior program.
Departments with fewer than 5 responses are shown but not compared.

Remove the facilitator's name from published comments and downloads,
replace the broken "Invalid Date" comment column with session dates,
and use plain "Recommendation Score" / "Satisfaction Ratings" wording
on all pages. Headline figures on the existing pages are unchanged.

Adds scripts/lds-survey/ build and QC scripts for future refreshes;
names to redact live in a git-ignored file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/lds-survey-dashboard/LDS_Survey_Export_Editable.xlsx
+++ b/static/lds-survey-dashboard/LDS_Survey_Export_Editable.xlsx
@@ -832,7 +832,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Sarah was one of the best presenters I have had at Notre Dame. Good work!</t>
+          <t>The facilitator was one of the best presenters I have had at Notre Dame. Good work!</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>While I like the content (and find it valuable) the format of a virtual discussion over the lunch hour is challenging. I found little value in the breakout rooms, and I would have preferred this meeting not take place over the lunch hour (usually when people like to actually use the time to eat and step away from their computers). I think it would have been more valuable to have a one-hour refresher (even over Zoom) NOT during lunch with Sarah facilitating the whole time (rather than using breakout rooms)</t>
+          <t>While I like the content (and find it valuable) the format of a virtual discussion over the lunch hour is challenging. I found little value in the breakout rooms, and I would have preferred this meeting not take place over the lunch hour (usually when people like to actually use the time to eat and step away from their computers). I think it would have been more valuable to have a one-hour refresher (even over Zoom) NOT during lunch with the facilitator leading the whole time (rather than using breakout rooms)</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>The format of this virtual breakout session and activity was not effective for retaining information. I would have preferred to spend the full 60 minutes learning from and listening to Sarah Turner. Asking participants to type out their notes and then listen to them being read aloud when rejoining the larger group was challenging and did not add value to the session.
+          <t>The format of this virtual breakout session and activity was not effective for retaining information. I would have preferred to spend the full 60 minutes learning from and listening to the facilitator. Asking participants to type out their notes and then listen to them being read aloud when rejoining the larger group was challenging and did not add value to the session.
  If this format continues in future sessions, I will likely opt out of participating.</t>
         </is>
       </c>
@@ -4097,7 +4097,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Thanks to Sarah and the planning team!!</t>
+          <t>Thanks to the facilitator and the planning team!!</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>I've really appreciated this series of trainings. Sarah is an engaging presenter and the hands on/discussion actitivities help us build relationships with other leaders and help make the sticky (meaning, it's memorable and actionable!). Personally, I need to work on implementing more of the practices and tools provided, especially the time management tools from this last session. Thank you!</t>
+          <t>I've really appreciated this series of trainings. The facilitator is an engaging presenter and the hands on/discussion actitivities help us build relationships with other leaders and help make the sticky (meaning, it's memorable and actionable!). Personally, I need to work on implementing more of the practices and tools provided, especially the time management tools from this last session. Thank you!</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>I've really appreciated this series. Thank you Sarah and the organizing team for putting it together.</t>
+          <t>I've really appreciated this series. Thank you to the facilitator and the organizing team for putting it together.</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Sarah is outstanding. She is incredibly easy to follow and listen to. I learned a lot from the courses. My only negative is that there were times where I felt like she was trying to cram too much content into the sessions.</t>
+          <t>The facilitator is outstanding. She is incredibly easy to follow and listen to. I learned a lot from the courses. My only negative is that there were times where I felt like she was trying to cram too much content into the sessions.</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5475,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sarah was one of the best presenters I have had at Notre Dame. Good work!</t>
+          <t>The facilitator was one of the best presenters I have had at Notre Dame. Good work!</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>While I like the content (and find it valuable) the format of a virtual discussion over the lunch hour is challenging. I found little value in the breakout rooms, and I would have preferred this meeting not take place over the lunch hour (usually when people like to actually use the time to eat and step away from their computers). I think it would have been more valuable to have a one-hour refresher (even over Zoom) NOT during lunch with Sarah facilitating the whole time (rather than using breakout rooms)</t>
+          <t>While I like the content (and find it valuable) the format of a virtual discussion over the lunch hour is challenging. I found little value in the breakout rooms, and I would have preferred this meeting not take place over the lunch hour (usually when people like to actually use the time to eat and step away from their computers). I think it would have been more valuable to have a one-hour refresher (even over Zoom) NOT during lunch with the facilitator leading the whole time (rather than using breakout rooms)</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6280,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>The format of this virtual breakout session and activity was not effective for retaining information. I would have preferred to spend the full 60 minutes learning from and listening to Sarah Turner. Asking participants to type out their notes and then listen to them being read aloud when rejoining the larger group was challenging and did not add value to the session.
+          <t>The format of this virtual breakout session and activity was not effective for retaining information. I would have preferred to spend the full 60 minutes learning from and listening to the facilitator. Asking participants to type out their notes and then listen to them being read aloud when rejoining the larger group was challenging and did not add value to the session.
  If this format continues in future sessions, I will likely opt out of participating.</t>
         </is>
       </c>
@@ -6304,7 +6304,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Thanks to Sarah and the planning team!!</t>
+          <t>Thanks to the facilitator and the planning team!!</t>
         </is>
       </c>
     </row>
@@ -6419,7 +6419,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>I've really appreciated this series of trainings. Sarah is an engaging presenter and the hands on/discussion actitivities help us build relationships with other leaders and help make the sticky (meaning, it's memorable and actionable!). Personally, I need to work on implementing more of the practices and tools provided, especially the time management tools from this last session. Thank you!</t>
+          <t>I've really appreciated this series of trainings. The facilitator is an engaging presenter and the hands on/discussion actitivities help us build relationships with other leaders and help make the sticky (meaning, it's memorable and actionable!). Personally, I need to work on implementing more of the practices and tools provided, especially the time management tools from this last session. Thank you!</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>I've really appreciated this series. Thank you Sarah and the organizing team for putting it together.</t>
+          <t>I've really appreciated this series. Thank you to the facilitator and the organizing team for putting it together.</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Sarah is outstanding. She is incredibly easy to follow and listen to. I learned a lot from the courses. My only negative is that there were times where I felt like she was trying to cram too much content into the sessions.</t>
+          <t>The facilitator is outstanding. She is incredibly easy to follow and listen to. I learned a lot from the courses. My only negative is that there were times where I felt like she was trying to cram too much content into the sessions.</t>
         </is>
       </c>
     </row>

</xml_diff>